<commit_message>
feat: enhance WorkReportTab with rich text editor and performance deadline logic
- Added rich text editor for report sections in WorkReportTab.
- Implemented dynamic deadline resolution based on performance window configurations.
- Updated form state management to accommodate new rich text fields.
- Introduced required sections banner to highlight mandatory fields in reports.
- Refactored existing fields to use new rich text component.
- Improved file upload handling and template download functionality.
- Added ManagerKpiApprovalScreen export in index file.
- Integrated Tailwind typography plugin for enhanced text styling.
</commit_message>
<xml_diff>
--- a/public/templates/kpi-okr-import-mau.xlsx
+++ b/public/templates/kpi-okr-import-mau.xlsx
@@ -3,8 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Import KPI-OKR" sheetId="1" r:id="rId1"/>
-    <sheet name="Hướng dẫn" sheetId="2" r:id="rId2"/>
+    <sheet name="KPI-OKR Import" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -398,21 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
-  <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="50.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="24.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:M3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -440,16 +425,19 @@
         <v>Chỉ số mục tiêu</v>
       </c>
       <c r="I1" t="str">
-        <v>BC KẾT QUẢ</v>
+        <v>Số liệu</v>
       </c>
       <c r="J1" t="str">
-        <v>Người đánh giá</v>
+        <v>Đơn vị</v>
       </c>
       <c r="K1" t="str">
-        <v>QL ĐÁNH GIÁ</v>
+        <v>Evidence</v>
       </c>
       <c r="L1" t="str">
-        <v>QL NHẬN XÉT</v>
+        <v>Tự đánh giá</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Tự nhận xét</v>
       </c>
     </row>
     <row r="2">
@@ -477,17 +465,20 @@
       <c r="H2">
         <v>100</v>
       </c>
-      <c r="I2" t="str">
-        <v/>
+      <c r="I2">
+        <v>50000000</v>
       </c>
       <c r="J2" t="str">
-        <v>Họ tên QL</v>
+        <v>VND</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>https://example.com/evidence</v>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>OK</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Đã hoàn thành mục tiêu</v>
       </c>
     </row>
     <row r="3">
@@ -519,72 +510,21 @@
         <v/>
       </c>
       <c r="J3" t="str">
-        <v>Họ tên QL</v>
+        <v/>
       </c>
       <c r="K3" t="str">
-        <v>OK</v>
+        <v/>
       </c>
       <c r="L3" t="str">
-        <v>Ghi chú tùy chọn</v>
+        <v>NOT</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Cần hỗ trợ thêm</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A8"/>
-  <cols>
-    <col min="1" max="1" width="92.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Hướng dẫn import KPI/OKR (khớp chức năng Upload trên HRM)</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>• Chọn đúng team và kỳ tháng/năm trên màn hình; hệ thống gán mọi dòng vào kỳ đó.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>• Cột bắt buộc: Nhân sự | Hạng mục (KPI hoặc OKR) | Nội dung KPI/OKRs.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>• Tên Nhân sự phải trùng họ tên (hoặc phần trước @ của email) trong danh sách team.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>• Ưu tiên: gõ Ưu tiên 1 … Ưu tiên 3 hoặc số 0–99.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>• Ngày set: yyyy-mm-dd hoặc số serial Excel. QL ĐÁNH GIÁ: OK hoặc NOT (có thể để trống).</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>• Mỗi dòng = một mục. Nội dung tối đa 500 ký tự. File .csv dùng cùng tiêu đề cột.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enhance KPI/OKR import templates and approval logic
- Updated CSV and XLSX templates for KPI/OKR imports to remove unnecessary fields and improve clarity.
- Refactored `generate-kpi-okr-template.mjs` to align with new template structure.
- Introduced `requiresKpiApproval` logic in various components to manage KPI approval workflows.
- Enhanced `HrOrgStructure` and `KpiOkrWorkspace` components to utilize the new approval flag.
- Updated tests to cover new approval logic and template changes.
</commit_message>
<xml_diff>
--- a/public/templates/kpi-okr-import-mau.xlsx
+++ b/public/templates/kpi-okr-import-mau.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="KPI-OKR Import" sheetId="1" r:id="rId1"/>
+    <sheet name="Import KPI-OKR" sheetId="1" r:id="rId1"/>
+    <sheet name="Hướng dẫn" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +398,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:L3"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,36 +422,33 @@
         <v>Tháng</v>
       </c>
       <c r="C1" t="str">
-        <v>Ngày set KPI/OKRs</v>
+        <v>Nhân sự</v>
       </c>
       <c r="D1" t="str">
-        <v>Nhân sự</v>
+        <v>Hạng mục</v>
       </c>
       <c r="E1" t="str">
-        <v>Hạng mục</v>
+        <v>Thứ tự ưu tiên</v>
       </c>
       <c r="F1" t="str">
-        <v>Thứ tự ưu tiên</v>
+        <v>Nội dung KPI/OKRs</v>
       </c>
       <c r="G1" t="str">
-        <v>Nội dung KPI/OKRs</v>
+        <v>Chỉ số mục tiêu</v>
       </c>
       <c r="H1" t="str">
-        <v>Chỉ số mục tiêu</v>
+        <v>Số liệu</v>
       </c>
       <c r="I1" t="str">
-        <v>Số liệu</v>
+        <v>Đơn vị</v>
       </c>
       <c r="J1" t="str">
-        <v>Đơn vị</v>
+        <v>Evidence</v>
       </c>
       <c r="K1" t="str">
-        <v>Evidence</v>
+        <v>Tự đánh giá</v>
       </c>
       <c r="L1" t="str">
-        <v>Tự đánh giá</v>
-      </c>
-      <c r="M1" t="str">
         <v>Tự nhận xét</v>
       </c>
     </row>
@@ -448,36 +460,33 @@
         <v>T3/2026</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-03-05</v>
+        <v>Nguyễn Văn A</v>
       </c>
       <c r="D2" t="str">
-        <v>Nguyễn Văn A</v>
+        <v>KPI</v>
       </c>
       <c r="E2" t="str">
-        <v>KPI</v>
+        <v>Ưu tiên 1</v>
       </c>
       <c r="F2" t="str">
-        <v>Ưu tiên 1</v>
-      </c>
-      <c r="G2" t="str">
         <v>Ví dụ: Hoàn thành chỉ tiêu doanh số tháng (sửa hoặc xóa dòng mẫu)</v>
       </c>
+      <c r="G2">
+        <v>100</v>
+      </c>
       <c r="H2">
-        <v>100</v>
-      </c>
-      <c r="I2">
         <v>50000000</v>
       </c>
+      <c r="I2" t="str">
+        <v>VND</v>
+      </c>
       <c r="J2" t="str">
-        <v>VND</v>
+        <v>https://example.com/evidence</v>
       </c>
       <c r="K2" t="str">
-        <v>https://example.com/evidence</v>
+        <v>OK</v>
       </c>
       <c r="L2" t="str">
-        <v>OK</v>
-      </c>
-      <c r="M2" t="str">
         <v>Đã hoàn thành mục tiêu</v>
       </c>
     </row>
@@ -489,22 +498,22 @@
         <v>T3/2026</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-03-05</v>
+        <v>Nguyễn Văn A</v>
       </c>
       <c r="D3" t="str">
-        <v>Nguyễn Văn A</v>
+        <v>OKR</v>
       </c>
       <c r="E3" t="str">
-        <v>OKR</v>
+        <v>Ưu tiên 2</v>
       </c>
       <c r="F3" t="str">
-        <v>Ưu tiên 2</v>
-      </c>
-      <c r="G3" t="str">
         <v>Ví dụ: Ra mắt tính năng X trong quý (tối đa 500 ký tự)</v>
       </c>
-      <c r="H3">
+      <c r="G3">
         <v>1</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
       </c>
       <c r="I3" t="str">
         <v/>
@@ -513,18 +522,69 @@
         <v/>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>NOT</v>
       </c>
       <c r="L3" t="str">
-        <v>NOT</v>
-      </c>
-      <c r="M3" t="str">
         <v>Cần hỗ trợ thêm</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A8"/>
+  <cols>
+    <col min="1" max="1" width="92.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Hướng dẫn import KPI/OKR (khớp chức năng Upload trên HRM)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>• Chọn đúng team và kỳ tháng/năm trên màn hình; hệ thống gán mọi dòng vào kỳ đó.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>• Cột bắt buộc: Nhân sự | Hạng mục (KPI hoặc OKR) | Nội dung KPI/OKRs.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>• Tên Nhân sự phải trùng họ tên (hoặc phần trước @ của email) trong danh sách team.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>• Ưu tiên: gõ Ưu tiên 1 … Ưu tiên 3 hoặc số 0–99.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>• Ngày xét được hệ thống tự lấy theo ngày tạo KPI/OKR. Tự đánh giá: OK hoặc NOT (có thể để trống).</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>• Mỗi dòng = một mục. Nội dung tối đa 500 ký tự. File .csv dùng cùng tiêu đề cột.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>